<commit_message>
finished ordering and BOM
</commit_message>
<xml_diff>
--- a/hospital_traversing_robot/BOM.xlsx
+++ b/hospital_traversing_robot/BOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -152,6 +152,12 @@
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approx </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Given </t>
   </si>
 </sst>
 </file>
@@ -579,7 +585,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr defaultColWidth="10.54296875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
@@ -682,13 +688,15 @@
       <c r="B5" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="12"/>
+      <c r="C5" s="12" t="n">
+        <v>20</v>
+      </c>
       <c r="D5" s="12" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="13" t="n">
         <f aca="false">C5*D5</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F5" s="14"/>
       <c r="G5" s="13"/>
@@ -835,14 +843,14 @@
         <v>18</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="D13" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" s="13" t="n">
         <f aca="false">C13*D13</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="G13" s="13"/>
     </row>
@@ -1028,14 +1036,14 @@
         <v>29</v>
       </c>
       <c r="C23" s="12" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D23" s="12" t="n">
         <v>1</v>
       </c>
       <c r="E23" s="13" t="n">
         <f aca="false">C23*D23</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G23" s="13"/>
     </row>
@@ -1104,14 +1112,14 @@
         <v>33</v>
       </c>
       <c r="C27" s="12" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="D27" s="12" t="n">
         <v>2</v>
       </c>
       <c r="E27" s="13" t="n">
         <f aca="false">C27*D27</f>
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="G27" s="13"/>
     </row>
@@ -1123,14 +1131,14 @@
         <v>34</v>
       </c>
       <c r="C28" s="12" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="D28" s="12" t="n">
         <v>1</v>
       </c>
       <c r="E28" s="13" t="n">
         <f aca="false">C28*D28</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="G28" s="13"/>
     </row>
@@ -1141,11 +1149,16 @@
       <c r="B29" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C29" s="12"/>
+      <c r="C29" s="12" t="n">
+        <v>10</v>
+      </c>
       <c r="D29" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="E29" s="13"/>
+      <c r="E29" s="13" t="n">
+        <f aca="false">C29*D29</f>
+        <v>10</v>
+      </c>
       <c r="G29" s="13"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1156,14 +1169,14 @@
         <v>36</v>
       </c>
       <c r="C30" s="12" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="D30" s="12" t="n">
         <v>4</v>
       </c>
       <c r="E30" s="13" t="n">
         <f aca="false">C30*D30</f>
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="G30" s="13"/>
     </row>
@@ -1240,14 +1253,14 @@
         <v>41</v>
       </c>
       <c r="C35" s="12" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="D35" s="5" t="n">
         <v>2</v>
       </c>
       <c r="E35" s="13" t="n">
         <f aca="false">C35*D35</f>
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="F35" s="14"/>
       <c r="G35" s="15"/>
@@ -1290,10 +1303,26 @@
       <c r="D39" s="25"/>
       <c r="E39" s="26" t="n">
         <f aca="false">SUM(E2:E38)</f>
-        <v>1792</v>
+        <v>2592</v>
       </c>
       <c r="F39" s="27"/>
       <c r="G39" s="23"/>
+    </row>
+    <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E41" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F41" s="1" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E42" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F42" s="1" t="n">
+        <v>5000</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>